<commit_message>
chore: cập nhật file seed danh sách người dùng và số liệu index GitNexus
</commit_message>
<xml_diff>
--- a/apps/api/prisma/initial-databases/betonghonglinh/data/Danh_sach_nguoi_dung.xlsx
+++ b/apps/api/prisma/initial-databases/betonghonglinh/data/Danh_sach_nguoi_dung.xlsx
@@ -397,50 +397,118 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>DANH SÁCH NGƯỜI DÙNG</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>STT</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Email</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Tên</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Vai trò</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Trạng thái</v>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>STT</v>
+      <c r="A3">
+        <v>1</v>
       </c>
       <c r="B3" t="str">
-        <v>Email</v>
+        <v>admin@ketoan.vn</v>
       </c>
       <c r="C3" t="str">
-        <v>Tên</v>
+        <v>Quản trị hệ thống</v>
       </c>
       <c r="D3" t="str">
-        <v>Vai trò</v>
+        <v>ADMIN</v>
       </c>
       <c r="E3" t="str">
-        <v>Trạng thái</v>
+        <v>Đang sử dụng</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="str">
-        <v>admin@ketoan.vn</v>
+        <v>ketoan@ketoan.vn</v>
       </c>
       <c r="C4" t="str">
-        <v>Quản trị hệ thống</v>
+        <v>Nguyễn Thị Hồng</v>
       </c>
       <c r="D4" t="str">
-        <v>ADMIN</v>
+        <v>KETOAN</v>
       </c>
       <c r="E4" t="str">
         <v>Đang sử dụng</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="str">
+        <v>thuquy@ketoan.vn</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Trần Văn Quý</v>
+      </c>
+      <c r="D5" t="str">
+        <v>THUQUY</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Đang sử dụng</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="str">
+        <v>viewer@ketoan.vn</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Lê Minh Viên</v>
+      </c>
+      <c r="D6" t="str">
+        <v>VIEWER</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Đang sử dụng</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" t="str">
+        <v>thutrang@ketoan.vn</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Phạm Thu Trang</v>
+      </c>
+      <c r="D7" t="str">
+        <v>KETOAN</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Ngừng sử dụng</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(api): bộ dữ liệu betonghonglinh chỉ còn 1 user admin
</commit_message>
<xml_diff>
--- a/apps/api/prisma/initial-databases/betonghonglinh/data/Danh_sach_nguoi_dung.xlsx
+++ b/apps/api/prisma/initial-databases/betonghonglinh/data/Danh_sach_nguoi_dung.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="DANH SÁCH NGƯỜI DÙNG" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -438,77 +438,9 @@
         <v>Đang sử dụng</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="str">
-        <v>ketoan@ketoan.vn</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Nguyễn Thị Hồng</v>
-      </c>
-      <c r="D4" t="str">
-        <v>KETOAN</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Đang sử dụng</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5" t="str">
-        <v>thuquy@ketoan.vn</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Trần Văn Quý</v>
-      </c>
-      <c r="D5" t="str">
-        <v>THUQUY</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Đang sử dụng</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>4</v>
-      </c>
-      <c r="B6" t="str">
-        <v>viewer@ketoan.vn</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Lê Minh Viên</v>
-      </c>
-      <c r="D6" t="str">
-        <v>VIEWER</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Đang sử dụng</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>5</v>
-      </c>
-      <c r="B7" t="str">
-        <v>thutrang@ketoan.vn</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Phạm Thu Trang</v>
-      </c>
-      <c r="D7" t="str">
-        <v>KETOAN</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Ngừng sử dụng</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>